<commit_message>
--cambios en el formato de la plantilla de informe de servicios de interior. Agregando: 1. Nombre de la empresa 2. Orden por número de cliente 2.1 Orden descendente por período
</commit_message>
<xml_diff>
--- a/Control de Facturas/Assets/Plantillas/Plantillas Pagos/INTERIOR.xlsx
+++ b/Control de Facturas/Assets/Plantillas/Plantillas Pagos/INTERIOR.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Programa Servicios Basicos\Control de Facturas\Assets\Plantillas\Plantillas Pagos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8937F1B-CD7A-46D5-8CEC-AB427895F20B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{348C55B7-EAF9-44A0-AB42-46BAC335C1B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15735" yWindow="930" windowWidth="15780" windowHeight="7785" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Informe de Pago Realizado" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Número de Cliente</t>
   </si>
@@ -61,6 +61,12 @@
   </si>
   <si>
     <t>Vencimiento Codigo de Autorizacion</t>
+  </si>
+  <si>
+    <t>Empresa</t>
+  </si>
+  <si>
+    <t>Periodo</t>
   </si>
 </sst>
 </file>
@@ -454,429 +460,442 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J65"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="13.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" style="3" customWidth="1"/>
-    <col min="2" max="3" width="13.28515625" style="3"/>
-    <col min="4" max="4" width="16.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.5703125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="13" style="3" customWidth="1"/>
+    <col min="3" max="3" width="16" style="3" customWidth="1"/>
+    <col min="4" max="4" width="8" style="3" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.28515625" style="3"/>
     <col min="6" max="6" width="16.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="13.28515625" style="3"/>
-    <col min="9" max="9" width="15" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="13.28515625" style="3"/>
+    <col min="7" max="7" width="13.28515625" style="3"/>
+    <col min="8" max="8" width="16.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.28515625" style="3"/>
+    <col min="11" max="11" width="15" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="13.28515625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C2" s="4"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E2" s="4"/>
       <c r="F2" s="5"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C3" s="4"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E3" s="4"/>
       <c r="F3" s="5"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C4" s="4"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C4" s="5"/>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C5" s="4"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C6" s="4"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C7" s="4"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E7" s="4"/>
       <c r="F7" s="5"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C8" s="4"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E8" s="4"/>
       <c r="F8" s="5"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C9" s="4"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E9" s="4"/>
       <c r="F9" s="5"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C10" s="4"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E10" s="4"/>
       <c r="F10" s="5"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C11" s="4"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E11" s="4"/>
       <c r="F11" s="5"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C12" s="4"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E12" s="4"/>
       <c r="F12" s="5"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C13" s="4"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E13" s="4"/>
       <c r="F13" s="5"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C14" s="4"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E14" s="4"/>
       <c r="F14" s="5"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C15" s="4"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E15" s="4"/>
       <c r="F15" s="5"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C16" s="4"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E16" s="4"/>
       <c r="F16" s="5"/>
-    </row>
-    <row r="17" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C17" s="4"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+    </row>
+    <row r="17" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E17" s="4"/>
       <c r="F17" s="5"/>
-    </row>
-    <row r="18" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C18" s="4"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
+    </row>
+    <row r="18" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E18" s="4"/>
       <c r="F18" s="5"/>
-    </row>
-    <row r="19" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C19" s="4"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+    </row>
+    <row r="19" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E19" s="4"/>
       <c r="F19" s="5"/>
-    </row>
-    <row r="20" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C20" s="4"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+    </row>
+    <row r="20" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E20" s="4"/>
       <c r="F20" s="5"/>
-    </row>
-    <row r="21" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C21" s="4"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+    </row>
+    <row r="21" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E21" s="4"/>
       <c r="F21" s="5"/>
-    </row>
-    <row r="22" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C22" s="4"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+    </row>
+    <row r="22" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E22" s="4"/>
       <c r="F22" s="5"/>
-    </row>
-    <row r="23" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C23" s="4"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+    </row>
+    <row r="23" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E23" s="4"/>
       <c r="F23" s="5"/>
-    </row>
-    <row r="24" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C24" s="4"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+    </row>
+    <row r="24" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E24" s="4"/>
       <c r="F24" s="5"/>
-    </row>
-    <row r="25" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C25" s="4"/>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+    </row>
+    <row r="25" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E25" s="4"/>
       <c r="F25" s="5"/>
-    </row>
-    <row r="26" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C26" s="4"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+    </row>
+    <row r="26" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E26" s="4"/>
       <c r="F26" s="5"/>
-    </row>
-    <row r="27" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C27" s="4"/>
-      <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+    </row>
+    <row r="27" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E27" s="4"/>
       <c r="F27" s="5"/>
-    </row>
-    <row r="28" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C28" s="4"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
+    </row>
+    <row r="28" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E28" s="4"/>
       <c r="F28" s="5"/>
-    </row>
-    <row r="29" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C29" s="4"/>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="5"/>
+    </row>
+    <row r="29" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E29" s="4"/>
       <c r="F29" s="5"/>
-    </row>
-    <row r="30" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C30" s="4"/>
-      <c r="D30" s="5"/>
-      <c r="E30" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+    </row>
+    <row r="30" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E30" s="4"/>
       <c r="F30" s="5"/>
-    </row>
-    <row r="31" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C31" s="4"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5"/>
+      <c r="G30" s="5"/>
+      <c r="H30" s="5"/>
+    </row>
+    <row r="31" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E31" s="4"/>
       <c r="F31" s="5"/>
-    </row>
-    <row r="32" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C32" s="4"/>
-      <c r="D32" s="5"/>
-      <c r="E32" s="5"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="5"/>
+    </row>
+    <row r="32" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E32" s="4"/>
       <c r="F32" s="5"/>
-    </row>
-    <row r="33" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C33" s="4"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
+    </row>
+    <row r="33" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E33" s="4"/>
       <c r="F33" s="5"/>
-    </row>
-    <row r="34" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C34" s="4"/>
-      <c r="D34" s="5"/>
-      <c r="E34" s="5"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+    </row>
+    <row r="34" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E34" s="4"/>
       <c r="F34" s="5"/>
-    </row>
-    <row r="35" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C35" s="4"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
+      <c r="G34" s="5"/>
+      <c r="H34" s="5"/>
+    </row>
+    <row r="35" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E35" s="4"/>
       <c r="F35" s="5"/>
-    </row>
-    <row r="36" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C36" s="4"/>
-      <c r="D36" s="5"/>
-      <c r="E36" s="5"/>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5"/>
+    </row>
+    <row r="36" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E36" s="4"/>
       <c r="F36" s="5"/>
-    </row>
-    <row r="37" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C37" s="4"/>
-      <c r="D37" s="5"/>
-      <c r="E37" s="5"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="5"/>
+    </row>
+    <row r="37" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E37" s="4"/>
       <c r="F37" s="5"/>
-    </row>
-    <row r="38" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C38" s="4"/>
-      <c r="D38" s="5"/>
-      <c r="E38" s="5"/>
+      <c r="G37" s="5"/>
+      <c r="H37" s="5"/>
+    </row>
+    <row r="38" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E38" s="4"/>
       <c r="F38" s="5"/>
-    </row>
-    <row r="39" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C39" s="4"/>
-      <c r="D39" s="5"/>
-      <c r="E39" s="5"/>
+      <c r="G38" s="5"/>
+      <c r="H38" s="5"/>
+    </row>
+    <row r="39" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E39" s="4"/>
       <c r="F39" s="5"/>
-    </row>
-    <row r="40" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C40" s="4"/>
-      <c r="D40" s="5"/>
-      <c r="E40" s="5"/>
+      <c r="G39" s="5"/>
+      <c r="H39" s="5"/>
+    </row>
+    <row r="40" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E40" s="4"/>
       <c r="F40" s="5"/>
-    </row>
-    <row r="41" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C41" s="4"/>
-      <c r="D41" s="5"/>
-      <c r="E41" s="5"/>
+      <c r="G40" s="5"/>
+      <c r="H40" s="5"/>
+    </row>
+    <row r="41" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E41" s="4"/>
       <c r="F41" s="5"/>
-    </row>
-    <row r="42" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C42" s="4"/>
-      <c r="D42" s="5"/>
-      <c r="E42" s="5"/>
+      <c r="G41" s="5"/>
+      <c r="H41" s="5"/>
+    </row>
+    <row r="42" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E42" s="4"/>
       <c r="F42" s="5"/>
-    </row>
-    <row r="43" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C43" s="4"/>
-      <c r="D43" s="5"/>
-      <c r="E43" s="5"/>
+      <c r="G42" s="5"/>
+      <c r="H42" s="5"/>
+    </row>
+    <row r="43" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E43" s="4"/>
       <c r="F43" s="5"/>
-    </row>
-    <row r="44" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C44" s="4"/>
-      <c r="D44" s="5"/>
-      <c r="E44" s="5"/>
+      <c r="G43" s="5"/>
+      <c r="H43" s="5"/>
+    </row>
+    <row r="44" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E44" s="4"/>
       <c r="F44" s="5"/>
-    </row>
-    <row r="45" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C45" s="4"/>
-      <c r="D45" s="5"/>
-      <c r="E45" s="5"/>
+      <c r="G44" s="5"/>
+      <c r="H44" s="5"/>
+    </row>
+    <row r="45" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E45" s="4"/>
       <c r="F45" s="5"/>
-    </row>
-    <row r="46" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C46" s="4"/>
-      <c r="D46" s="5"/>
-      <c r="E46" s="5"/>
+      <c r="G45" s="5"/>
+      <c r="H45" s="5"/>
+    </row>
+    <row r="46" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E46" s="4"/>
       <c r="F46" s="5"/>
-    </row>
-    <row r="47" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C47" s="4"/>
-      <c r="D47" s="5"/>
-      <c r="E47" s="5"/>
+      <c r="G46" s="5"/>
+      <c r="H46" s="5"/>
+    </row>
+    <row r="47" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E47" s="4"/>
       <c r="F47" s="5"/>
-    </row>
-    <row r="48" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C48" s="4"/>
-      <c r="D48" s="5"/>
-      <c r="E48" s="5"/>
+      <c r="G47" s="5"/>
+      <c r="H47" s="5"/>
+    </row>
+    <row r="48" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E48" s="4"/>
       <c r="F48" s="5"/>
-    </row>
-    <row r="49" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C49" s="4"/>
-      <c r="D49" s="5"/>
-      <c r="E49" s="5"/>
+      <c r="G48" s="5"/>
+      <c r="H48" s="5"/>
+    </row>
+    <row r="49" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E49" s="4"/>
       <c r="F49" s="5"/>
-    </row>
-    <row r="50" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C50" s="4"/>
-      <c r="D50" s="5"/>
-      <c r="E50" s="5"/>
+      <c r="G49" s="5"/>
+      <c r="H49" s="5"/>
+    </row>
+    <row r="50" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E50" s="4"/>
       <c r="F50" s="5"/>
-    </row>
-    <row r="51" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C51" s="4"/>
-      <c r="D51" s="5"/>
-      <c r="E51" s="5"/>
+      <c r="G50" s="5"/>
+      <c r="H50" s="5"/>
+    </row>
+    <row r="51" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E51" s="4"/>
       <c r="F51" s="5"/>
-    </row>
-    <row r="52" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C52" s="4"/>
-      <c r="D52" s="5"/>
-      <c r="E52" s="5"/>
+      <c r="G51" s="5"/>
+      <c r="H51" s="5"/>
+    </row>
+    <row r="52" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E52" s="4"/>
       <c r="F52" s="5"/>
-    </row>
-    <row r="53" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C53" s="4"/>
-      <c r="D53" s="5"/>
-      <c r="E53" s="5"/>
+      <c r="G52" s="5"/>
+      <c r="H52" s="5"/>
+    </row>
+    <row r="53" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E53" s="4"/>
       <c r="F53" s="5"/>
-    </row>
-    <row r="54" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C54" s="4"/>
-      <c r="D54" s="5"/>
-      <c r="E54" s="5"/>
+      <c r="G53" s="5"/>
+      <c r="H53" s="5"/>
+    </row>
+    <row r="54" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E54" s="4"/>
       <c r="F54" s="5"/>
-    </row>
-    <row r="55" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C55" s="4"/>
-      <c r="D55" s="5"/>
-      <c r="E55" s="5"/>
+      <c r="G54" s="5"/>
+      <c r="H54" s="5"/>
+    </row>
+    <row r="55" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E55" s="4"/>
       <c r="F55" s="5"/>
-    </row>
-    <row r="56" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C56" s="4"/>
-      <c r="D56" s="5"/>
-      <c r="E56" s="5"/>
+      <c r="G55" s="5"/>
+      <c r="H55" s="5"/>
+    </row>
+    <row r="56" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E56" s="4"/>
       <c r="F56" s="5"/>
-    </row>
-    <row r="57" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C57" s="4"/>
-      <c r="D57" s="5"/>
-      <c r="E57" s="5"/>
+      <c r="G56" s="5"/>
+      <c r="H56" s="5"/>
+    </row>
+    <row r="57" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E57" s="4"/>
       <c r="F57" s="5"/>
-    </row>
-    <row r="58" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C58" s="4"/>
-      <c r="D58" s="5"/>
-      <c r="E58" s="5"/>
+      <c r="G57" s="5"/>
+      <c r="H57" s="5"/>
+    </row>
+    <row r="58" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E58" s="4"/>
       <c r="F58" s="5"/>
-    </row>
-    <row r="59" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C59" s="4"/>
-      <c r="D59" s="5"/>
-      <c r="E59" s="5"/>
+      <c r="G58" s="5"/>
+      <c r="H58" s="5"/>
+    </row>
+    <row r="59" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E59" s="4"/>
       <c r="F59" s="5"/>
-    </row>
-    <row r="60" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C60" s="4"/>
-      <c r="D60" s="5"/>
-      <c r="E60" s="5"/>
+      <c r="G59" s="5"/>
+      <c r="H59" s="5"/>
+    </row>
+    <row r="60" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E60" s="4"/>
       <c r="F60" s="5"/>
-    </row>
-    <row r="61" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C61" s="4"/>
-      <c r="D61" s="5"/>
-      <c r="E61" s="5"/>
+      <c r="G60" s="5"/>
+      <c r="H60" s="5"/>
+    </row>
+    <row r="61" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E61" s="4"/>
       <c r="F61" s="5"/>
-    </row>
-    <row r="62" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C62" s="4"/>
-      <c r="D62" s="5"/>
-      <c r="E62" s="5"/>
+      <c r="G61" s="5"/>
+      <c r="H61" s="5"/>
+    </row>
+    <row r="62" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E62" s="4"/>
       <c r="F62" s="5"/>
-    </row>
-    <row r="63" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C63" s="4"/>
-      <c r="D63" s="5"/>
-      <c r="E63" s="5"/>
+      <c r="G62" s="5"/>
+      <c r="H62" s="5"/>
+    </row>
+    <row r="63" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E63" s="4"/>
       <c r="F63" s="5"/>
-    </row>
-    <row r="65" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F65" s="6"/>
+      <c r="G63" s="5"/>
+      <c r="H63" s="5"/>
+    </row>
+    <row r="65" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H65" s="6"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J63">
-    <sortCondition ref="A2:A63"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:L63">
+    <sortCondition ref="B2:B63"/>
   </sortState>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="30" orientation="portrait" r:id="rId1"/>

</xml_diff>